<commit_message>
Fix 2026 report date for July 8 update
</commit_message>
<xml_diff>
--- a/每日振幅统计_2026.xlsx
+++ b/每日振幅统计_2026.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R428509857a6b4527"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="Re57a2ad2bd1b4fb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R23abfd971ea24e2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="R9f2668ea5e994d93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Re582d1f3fbb94019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R529d0f7e58f943c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="R86f0ed9783174dc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R952fc92eaae54a6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" r:id="R6533aed68dd246ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证1000" sheetId="2" r:id="R7bf3e5c015bd4d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="3" r:id="R8e992f62f35c4a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="上证指数" sheetId="4" r:id="Rb8515c959fb94a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM主力" sheetId="5" r:id="Rda7d208b900f4d35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC主力" sheetId="6" r:id="R31ad5425031f4b39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IF主力" sheetId="7" r:id="Rf5e0c8cbe40049d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IH主力" sheetId="8" r:id="R896fd459e8b843ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -699,7 +699,7 @@
         <x:v>2026-01-01</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>2026-07-09</x:v>
+        <x:v>2026-07-08</x:v>
       </x:c>
       <x:c r="D13" s="14" t="str">
         <x:v>数据源</x:v>

</xml_diff>